<commit_message>
Fase 1 en una sola carpeta, imagenes por producto y validacion de la Fase 2
- Fase 1: queda solo lo entregado el 19-09 (se quitan la copia descargada
  de Drive y las plantillas de trabajo; siguen en el historial).
- Imagenes de producto: una ilustracion propia por producto en vez de la
  rueda del logo.
- Excel: columna Contacto en la hoja de proveedores.
- _Referencia/validacion_enunciado_fase2.md: cada requisito del enunciado
  para la Fase 2, donde se cubre y su estado.
</commit_message>
<xml_diff>
--- a/Entrega_Fase2_Grupo14/3_Archivos_Datos/RutaMoto_datos_maestros_Fase2.xlsx
+++ b/Entrega_Fase2_Grupo14/3_Archivos_Datos/RutaMoto_datos_maestros_Fase2.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1_Productos'!$A$1:$J$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2_Existencias_iniciales'!$A$1:$F$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3_Reglas_reabastecimiento'!$A$1:$F$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4_Proveedores'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4_Proveedores'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5_Contactos_proveedores'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_Productos_por_proveedor'!$A$1:$F$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7_Clientes'!$A$1:$H$36</definedName>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="478">
   <si>
     <t>RutaMoto · Datos maestros para la carga en Odoo · Fase 2 · Grupo 14</t>
   </si>
@@ -489,6 +489,9 @@
     <t>Plazo de pago del proveedor</t>
   </si>
   <si>
+    <t>Contacto (informativo)</t>
+  </si>
+  <si>
     <t>Qué provee (informativo)</t>
   </si>
   <si>
@@ -513,6 +516,9 @@
     <t>30 días</t>
   </si>
   <si>
+    <t>Rosa Elena Batres, Ejecutiva de ventas</t>
+  </si>
+  <si>
     <t>Crédito 30 días</t>
   </si>
   <si>
@@ -528,6 +534,9 @@
     <t>Zona industrial, bodega 4</t>
   </si>
   <si>
+    <t>Mario Roberto Ixcot, Asesor comercial</t>
+  </si>
+  <si>
     <t>Distribuidora Llantera del Sur</t>
   </si>
   <si>
@@ -543,6 +552,9 @@
     <t>50% anticipo, 50% contra entrega</t>
   </si>
   <si>
+    <t>Claudia Patricia Monzón, Encargada de cuentas</t>
+  </si>
+  <si>
     <t>Grupo Eléctrico Moto GT</t>
   </si>
   <si>
@@ -558,6 +570,9 @@
     <t>15 días</t>
   </si>
   <si>
+    <t>Juan Carlos Pac, Vendedor de ruta</t>
+  </si>
+  <si>
     <t>Crédito 15 días</t>
   </si>
   <si>
@@ -574,6 +589,9 @@
   </si>
   <si>
     <t>45 días</t>
+  </si>
+  <si>
+    <t>Silvia Marisol Recinos, Gerente de ventas</t>
   </si>
   <si>
     <t>Crédito 45 días</t>
@@ -2022,196 +2040,196 @@
   <sheetData>
     <row r="1" spans="1:4" ht="32" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="6" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="6" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="6" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="6" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>29</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="6" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="6" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="6" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="6" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="6" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>150</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="6" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="6" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="6" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="6" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>144</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -2231,15 +2249,15 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>18</v>
@@ -2250,7 +2268,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="B4" s="9">
         <v>30</v>
@@ -2265,7 +2283,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="B5" s="9">
         <v>5</v>
@@ -2280,7 +2298,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="B6" s="9">
         <v>35</v>
@@ -2295,7 +2313,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="B7" s="9">
         <v>12</v>
@@ -2310,7 +2328,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="B8" s="9">
         <v>11</v>
@@ -2325,7 +2343,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="9" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="B9" s="9">
         <v>7</v>
@@ -2340,7 +2358,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="9" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="B10" s="9">
         <v>5</v>
@@ -2355,7 +2373,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="11" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="B11" s="11">
         <v>38096</v>
@@ -2370,73 +2388,73 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="3" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="3" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="9" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="9" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="9" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="9" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="3" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
   </sheetData>
@@ -4776,7 +4794,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.7109375" customWidth="1"/>
@@ -4786,11 +4804,12 @@
     <col min="5" max="5" width="26.7109375" customWidth="1"/>
     <col min="6" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="30.7109375" customWidth="1"/>
-    <col min="9" max="9" width="28.7109375" customWidth="1"/>
-    <col min="10" max="10" width="30.7109375" customWidth="1"/>
+    <col min="9" max="9" width="34.7109375" customWidth="1"/>
+    <col min="10" max="10" width="28.7109375" customWidth="1"/>
+    <col min="11" max="11" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="32" customHeight="1">
+    <row r="1" spans="1:11" ht="32" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>25</v>
       </c>
@@ -4821,169 +4840,187 @@
       <c r="J1" s="5" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H2" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="I2" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="J2" s="8" t="s">
+      <c r="G3" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="6" t="s">
+      <c r="I3" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K3" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="H3" s="6" t="s">
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="I3" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>157</v>
-      </c>
       <c r="G4" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="I4" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4" s="8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="I5" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5" s="8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="I6" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>180</v>
+      <c r="K6" s="8" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:K6"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5005,10 +5042,10 @@
         <v>25</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>145</v>
@@ -5019,87 +5056,87 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="6" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="6" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="6" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="6" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="6" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -5121,27 +5158,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="32" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>130</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>138</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>35</v>
@@ -5161,7 +5198,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>40</v>
@@ -5181,7 +5218,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>43</v>
@@ -5201,7 +5238,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>46</v>
@@ -5221,7 +5258,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>49</v>
@@ -5241,7 +5278,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>52</v>
@@ -5261,7 +5298,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>55</v>
@@ -5281,7 +5318,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>59</v>
@@ -5301,7 +5338,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>62</v>
@@ -5321,7 +5358,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>65</v>
@@ -5341,7 +5378,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>68</v>
@@ -5361,7 +5398,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>71</v>
@@ -5381,7 +5418,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>74</v>
@@ -5401,7 +5438,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>78</v>
@@ -5421,7 +5458,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>81</v>
@@ -5441,7 +5478,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>84</v>
@@ -5461,7 +5498,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>87</v>
@@ -5481,7 +5518,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>90</v>
@@ -5501,7 +5538,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>93</v>
@@ -5521,7 +5558,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>97</v>
@@ -5541,7 +5578,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>100</v>
@@ -5561,7 +5598,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>103</v>
@@ -5581,7 +5618,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>106</v>
@@ -5601,7 +5638,7 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>109</v>
@@ -5621,7 +5658,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>112</v>
@@ -5641,7 +5678,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>116</v>
@@ -5661,7 +5698,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>119</v>
@@ -5681,7 +5718,7 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>122</v>
@@ -5701,7 +5738,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>125</v>
@@ -5721,7 +5758,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>128</v>
@@ -5767,7 +5804,7 @@
         <v>144</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>145</v>
@@ -5787,912 +5824,912 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="6" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="6" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="6" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="6" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="6" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="6" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="6" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="6" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="6" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="6" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="6" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="6" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="6" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="6" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="6" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="6" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="6" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="6" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="6" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="6" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="6" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="6" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="6" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="6" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="6" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="6" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="6" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="6" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="6" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="6" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="6" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -6721,17 +6758,17 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="12" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -6739,42 +6776,42 @@
         <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>146</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="6" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="G6" s="6">
         <v>6</v>
@@ -6782,7 +6819,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="12" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -6793,7 +6830,7 @@
         <v>25</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>27</v>
@@ -6802,24 +6839,24 @@
         <v>28</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="6" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D10" s="7">
         <v>450</v>
@@ -6839,13 +6876,13 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="6" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D11" s="7">
         <v>220</v>
@@ -6865,13 +6902,13 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="6" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D12" s="7">
         <v>95</v>
@@ -6891,13 +6928,13 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="6" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>372</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>366</v>
       </c>
       <c r="D13" s="7">
         <v>120</v>
@@ -6917,13 +6954,13 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="6" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D14" s="7">
         <v>140</v>
@@ -6943,13 +6980,13 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="6" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D15" s="7">
         <v>185</v>
@@ -6969,7 +7006,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="12" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -6977,13 +7014,13 @@
         <v>25</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>146</v>
@@ -6997,122 +7034,122 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="6" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="6" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="6" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="6" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="6" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="3" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="D25" s="11">
         <v>6904</v>

</xml_diff>